<commit_message>
Rerun analysis to reflect volatility of throughput, and reduce models tested to 3
</commit_message>
<xml_diff>
--- a/results/03_lead_lag_deconvolution/03_lead_lag_deconvolution.xlsx
+++ b/results/03_lead_lag_deconvolution/03_lead_lag_deconvolution.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Table_of_Contents" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Section_4B_Lead_Lag_Arrival_Dec" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_of_Contents" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Section_4B_Lead_Lag_Arrival_Dec" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Section_4B_Lead_Lag_Arrival_Dec'!$A$1:$F$7</definedName>
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>6</v>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -644,158 +644,184 @@
       </c>
     </row>
     <row r="2" ht="19" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Contemporaneous Departures (t)</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lag t-1 (1 hr post-departure)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>-1 hours (Post-Departure Hour)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1987</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.0395</v>
+      </c>
+      <c r="E2" t="n">
+        <v>16.06</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>-65.9% vs Baseline (Spurious Lag)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="19" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Same-Hour Departure t (Gate departure)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>0 hours (Takeoff Hour)</t>
         </is>
       </c>
-      <c r="C2" s="10" t="n">
-        <v>0.4459</v>
-      </c>
-      <c r="D2" s="11" t="n">
-        <v>0.1988</v>
-      </c>
-      <c r="E2" s="10" t="n">
-        <v>38.42</v>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>Baseline (Status Quo)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="19" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Lead Horizon t+1</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="C3" t="n">
+        <v>0.3403</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.1158</v>
+      </c>
+      <c r="E3" t="n">
+        <v>27.49</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Baseline (Unshifted Same-Hour Schedule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="19" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lead Horizon t+1 (1 hr pre-departure)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>1 hour pre-departure</t>
         </is>
       </c>
-      <c r="C3" s="10" t="n">
-        <v>0.6102</v>
-      </c>
-      <c r="D3" s="11" t="n">
-        <v>0.3723</v>
-      </c>
-      <c r="E3" s="10" t="n">
-        <v>62.15</v>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>+87.3% vs Baseline</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="19" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Lead Horizon t+2 (Peak Window)</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>2 hours pre-departure</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="n">
-        <v>0.6367</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>0.4054</v>
-      </c>
-      <c r="E4" s="10" t="n">
+      <c r="C4" t="n">
+        <v>0.4913</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.2413</v>
+      </c>
+      <c r="E4" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>+108.4% vs Baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="19" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lead Horizon t+2 (2 hr pre-departure)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2 hours pre-departure (Modal Window)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.4876</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.2378</v>
+      </c>
+      <c r="E5" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+105.4% vs Baseline (Global Peak)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Lead Horizon t+3 (3 hr pre-departure)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3 hours pre-departure</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.1444</v>
+      </c>
+      <c r="E6" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+24.7% vs Baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="19" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Convolved Passenger Show-Up Curve</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Distributed across t+1 to t+3</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.6985</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.4878</v>
+      </c>
+      <c r="E7" t="n">
         <v>74.98</v>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>+103.9% vs Baseline (Global Peak)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="19" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Lead Horizon t+3</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>3 hours pre-departure</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="n">
-        <v>0.5744</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>0.3299</v>
-      </c>
-      <c r="E5" s="10" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>+65.9% vs Baseline</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="19" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Continuous Convolved Lead Demand</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Distributed across t+1 to t+3</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>0.6985</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>0.4878</v>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>74.98</v>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>+145.4% vs Baseline</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="19" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Convolved Demand * T-100 Load Factor</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>+321.2% vs Baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Show-Up Curve * T-100 Load Factor</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Continuous with Carrier Load Factor</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C8" t="n">
         <v>0.7060999999999999</v>
       </c>
-      <c r="D7" s="11" t="n">
+      <c r="D8" t="n">
         <v>0.4985</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E8" t="n">
         <v>90.56</v>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>+150.8% vs Baseline</t>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+330.5% vs Baseline</t>
         </is>
       </c>
     </row>

</xml_diff>